<commit_message>
Filling the missing series number in the data field Team Number
</commit_message>
<xml_diff>
--- a/Data/WC2026_data.xlsx
+++ b/Data/WC2026_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sabee/Desktop/WC2026_Objective 2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/exwhyzed/github/WC2026_Objective-2/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B185040-5ECC-DF49-A904-74F1A13DD0E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99F17262-8924-3048-9E4F-A8A05A587266}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17940" activeTab="1" xr2:uid="{6D8C40B8-B365-E74B-851C-CDB1A87B4DC4}"/>
   </bookViews>
@@ -16105,6 +16105,9 @@
       </c>
     </row>
     <row r="50" spans="1:5">
+      <c r="A50">
+        <v>49</v>
+      </c>
       <c r="B50" t="s">
         <v>355</v>
       </c>
@@ -16119,6 +16122,9 @@
       </c>
     </row>
     <row r="51" spans="1:5">
+      <c r="A51">
+        <v>50</v>
+      </c>
       <c r="B51" t="s">
         <v>357</v>
       </c>
@@ -16133,6 +16139,9 @@
       </c>
     </row>
     <row r="52" spans="1:5">
+      <c r="A52">
+        <v>51</v>
+      </c>
       <c r="B52" t="s">
         <v>358</v>
       </c>
@@ -16147,6 +16156,9 @@
       </c>
     </row>
     <row r="53" spans="1:5">
+      <c r="A53">
+        <v>52</v>
+      </c>
       <c r="B53" t="s">
         <v>359</v>
       </c>
@@ -16161,6 +16173,9 @@
       </c>
     </row>
     <row r="54" spans="1:5">
+      <c r="A54">
+        <v>53</v>
+      </c>
       <c r="B54" t="s">
         <v>360</v>
       </c>
@@ -16175,6 +16190,9 @@
       </c>
     </row>
     <row r="55" spans="1:5">
+      <c r="A55">
+        <v>54</v>
+      </c>
       <c r="B55" t="s">
         <v>361</v>
       </c>
@@ -16189,6 +16207,9 @@
       </c>
     </row>
     <row r="56" spans="1:5">
+      <c r="A56">
+        <v>55</v>
+      </c>
       <c r="B56" t="s">
         <v>362</v>
       </c>
@@ -16203,6 +16224,9 @@
       </c>
     </row>
     <row r="57" spans="1:5">
+      <c r="A57">
+        <v>56</v>
+      </c>
       <c r="B57" t="s">
         <v>363</v>
       </c>
@@ -16217,6 +16241,9 @@
       </c>
     </row>
     <row r="58" spans="1:5">
+      <c r="A58">
+        <v>57</v>
+      </c>
       <c r="B58" t="s">
         <v>364</v>
       </c>
@@ -16231,6 +16258,9 @@
       </c>
     </row>
     <row r="59" spans="1:5">
+      <c r="A59">
+        <v>58</v>
+      </c>
       <c r="B59" t="s">
         <v>365</v>
       </c>
@@ -16245,6 +16275,9 @@
       </c>
     </row>
     <row r="60" spans="1:5">
+      <c r="A60">
+        <v>59</v>
+      </c>
       <c r="B60" t="s">
         <v>366</v>
       </c>
@@ -16259,6 +16292,9 @@
       </c>
     </row>
     <row r="61" spans="1:5">
+      <c r="A61">
+        <v>60</v>
+      </c>
       <c r="B61" t="s">
         <v>367</v>
       </c>
@@ -16273,6 +16309,9 @@
       </c>
     </row>
     <row r="62" spans="1:5">
+      <c r="A62">
+        <v>61</v>
+      </c>
       <c r="B62" t="s">
         <v>368</v>
       </c>
@@ -16287,6 +16326,9 @@
       </c>
     </row>
     <row r="63" spans="1:5">
+      <c r="A63">
+        <v>62</v>
+      </c>
       <c r="B63" t="s">
         <v>369</v>
       </c>
@@ -16301,6 +16343,9 @@
       </c>
     </row>
     <row r="64" spans="1:5">
+      <c r="A64">
+        <v>63</v>
+      </c>
       <c r="B64" t="s">
         <v>370</v>
       </c>
@@ -16314,7 +16359,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="65" spans="2:5">
+    <row r="65" spans="1:5">
+      <c r="A65">
+        <v>64</v>
+      </c>
       <c r="B65" t="s">
         <v>371</v>
       </c>
@@ -16328,7 +16376,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="66" spans="2:5">
+    <row r="66" spans="1:5">
+      <c r="A66">
+        <v>65</v>
+      </c>
       <c r="B66" t="s">
         <v>372</v>
       </c>
@@ -16342,7 +16393,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="67" spans="2:5">
+    <row r="67" spans="1:5">
+      <c r="A67">
+        <v>66</v>
+      </c>
       <c r="B67" t="s">
         <v>373</v>
       </c>
@@ -16356,7 +16410,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="68" spans="2:5">
+    <row r="68" spans="1:5">
+      <c r="A68">
+        <v>67</v>
+      </c>
       <c r="B68" t="s">
         <v>374</v>
       </c>
@@ -16370,7 +16427,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="69" spans="2:5">
+    <row r="69" spans="1:5">
+      <c r="A69">
+        <v>68</v>
+      </c>
       <c r="B69" t="s">
         <v>375</v>
       </c>
@@ -16384,7 +16444,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="70" spans="2:5">
+    <row r="70" spans="1:5">
+      <c r="A70">
+        <v>69</v>
+      </c>
       <c r="B70" t="s">
         <v>376</v>
       </c>
@@ -16398,7 +16461,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="71" spans="2:5">
+    <row r="71" spans="1:5">
+      <c r="A71">
+        <v>70</v>
+      </c>
       <c r="B71" t="s">
         <v>377</v>
       </c>
@@ -16412,7 +16478,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="72" spans="2:5">
+    <row r="72" spans="1:5">
+      <c r="A72">
+        <v>71</v>
+      </c>
       <c r="B72" t="s">
         <v>378</v>
       </c>
@@ -16426,7 +16495,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="73" spans="2:5">
+    <row r="73" spans="1:5">
+      <c r="A73">
+        <v>72</v>
+      </c>
       <c r="B73" t="s">
         <v>379</v>
       </c>
@@ -16440,7 +16512,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="74" spans="2:5">
+    <row r="74" spans="1:5">
+      <c r="A74">
+        <v>73</v>
+      </c>
       <c r="B74" t="s">
         <v>380</v>
       </c>
@@ -16454,7 +16529,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="75" spans="2:5">
+    <row r="75" spans="1:5">
+      <c r="A75">
+        <v>74</v>
+      </c>
       <c r="B75" t="s">
         <v>380</v>
       </c>
@@ -16468,7 +16546,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="76" spans="2:5">
+    <row r="76" spans="1:5">
+      <c r="A76">
+        <v>75</v>
+      </c>
       <c r="B76" t="s">
         <v>381</v>
       </c>
@@ -16482,7 +16563,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="77" spans="2:5">
+    <row r="77" spans="1:5">
+      <c r="A77">
+        <v>76</v>
+      </c>
       <c r="B77" t="s">
         <v>382</v>
       </c>
@@ -16496,7 +16580,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="78" spans="2:5">
+    <row r="78" spans="1:5">
+      <c r="A78">
+        <v>77</v>
+      </c>
       <c r="B78" t="s">
         <v>383</v>
       </c>
@@ -16510,7 +16597,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="79" spans="2:5">
+    <row r="79" spans="1:5">
+      <c r="A79">
+        <v>78</v>
+      </c>
       <c r="B79" t="s">
         <v>384</v>
       </c>
@@ -16524,7 +16614,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="80" spans="2:5">
+    <row r="80" spans="1:5">
+      <c r="A80">
+        <v>79</v>
+      </c>
       <c r="B80" t="s">
         <v>385</v>
       </c>
@@ -16538,7 +16631,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="81" spans="2:5">
+    <row r="81" spans="1:5">
+      <c r="A81">
+        <v>80</v>
+      </c>
       <c r="B81" t="s">
         <v>386</v>
       </c>
@@ -16552,7 +16648,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="82" spans="2:5">
+    <row r="82" spans="1:5">
+      <c r="A82">
+        <v>81</v>
+      </c>
       <c r="B82" t="s">
         <v>387</v>
       </c>
@@ -16566,7 +16665,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="83" spans="2:5">
+    <row r="83" spans="1:5">
+      <c r="A83">
+        <v>82</v>
+      </c>
       <c r="B83" t="s">
         <v>388</v>
       </c>
@@ -16580,7 +16682,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="84" spans="2:5">
+    <row r="84" spans="1:5">
+      <c r="A84">
+        <v>83</v>
+      </c>
       <c r="B84" t="s">
         <v>389</v>
       </c>
@@ -16594,7 +16699,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="85" spans="2:5">
+    <row r="85" spans="1:5">
+      <c r="A85">
+        <v>84</v>
+      </c>
       <c r="B85" t="s">
         <v>390</v>
       </c>
@@ -16608,7 +16716,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="86" spans="2:5">
+    <row r="86" spans="1:5">
+      <c r="A86">
+        <v>85</v>
+      </c>
       <c r="B86" t="s">
         <v>391</v>
       </c>
@@ -16622,7 +16733,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="87" spans="2:5">
+    <row r="87" spans="1:5">
+      <c r="A87">
+        <v>86</v>
+      </c>
       <c r="B87" t="s">
         <v>392</v>
       </c>
@@ -16636,7 +16750,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="88" spans="2:5">
+    <row r="88" spans="1:5">
+      <c r="A88">
+        <v>87</v>
+      </c>
       <c r="B88" t="s">
         <v>393</v>
       </c>
@@ -16650,7 +16767,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="89" spans="2:5">
+    <row r="89" spans="1:5">
+      <c r="A89">
+        <v>88</v>
+      </c>
       <c r="B89" t="s">
         <v>394</v>
       </c>
@@ -16664,7 +16784,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="90" spans="2:5">
+    <row r="90" spans="1:5">
+      <c r="A90">
+        <v>89</v>
+      </c>
       <c r="B90" t="s">
         <v>395</v>
       </c>
@@ -16678,7 +16801,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="91" spans="2:5">
+    <row r="91" spans="1:5">
+      <c r="A91">
+        <v>90</v>
+      </c>
       <c r="B91" t="s">
         <v>396</v>
       </c>
@@ -16692,7 +16818,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="92" spans="2:5">
+    <row r="92" spans="1:5">
+      <c r="A92">
+        <v>91</v>
+      </c>
       <c r="B92" t="s">
         <v>397</v>
       </c>
@@ -16706,7 +16835,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="93" spans="2:5">
+    <row r="93" spans="1:5">
+      <c r="A93">
+        <v>92</v>
+      </c>
       <c r="B93" t="s">
         <v>398</v>
       </c>
@@ -16720,7 +16852,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="94" spans="2:5">
+    <row r="94" spans="1:5">
+      <c r="A94">
+        <v>93</v>
+      </c>
       <c r="B94" t="s">
         <v>399</v>
       </c>
@@ -16734,7 +16869,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="95" spans="2:5">
+    <row r="95" spans="1:5">
+      <c r="A95">
+        <v>94</v>
+      </c>
       <c r="B95" t="s">
         <v>400</v>
       </c>
@@ -16748,7 +16886,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="96" spans="2:5">
+    <row r="96" spans="1:5">
+      <c r="A96">
+        <v>95</v>
+      </c>
       <c r="B96" t="s">
         <v>401</v>
       </c>
@@ -16762,7 +16903,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="97" spans="2:5">
+    <row r="97" spans="1:5">
+      <c r="A97">
+        <v>96</v>
+      </c>
       <c r="B97" t="s">
         <v>402</v>
       </c>
@@ -16776,7 +16920,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="98" spans="2:5">
+    <row r="98" spans="1:5">
+      <c r="A98">
+        <v>97</v>
+      </c>
       <c r="B98" t="s">
         <v>403</v>
       </c>
@@ -16790,7 +16937,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="99" spans="2:5">
+    <row r="99" spans="1:5">
+      <c r="A99">
+        <v>98</v>
+      </c>
       <c r="B99" t="s">
         <v>404</v>
       </c>
@@ -16804,7 +16954,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="100" spans="2:5">
+    <row r="100" spans="1:5">
+      <c r="A100">
+        <v>99</v>
+      </c>
       <c r="B100" t="s">
         <v>405</v>
       </c>
@@ -16818,7 +16971,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="101" spans="2:5">
+    <row r="101" spans="1:5">
+      <c r="A101">
+        <v>100</v>
+      </c>
       <c r="B101" t="s">
         <v>406</v>
       </c>
@@ -16832,7 +16988,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="102" spans="2:5">
+    <row r="102" spans="1:5">
+      <c r="A102">
+        <v>101</v>
+      </c>
       <c r="B102" t="s">
         <v>407</v>
       </c>
@@ -16846,7 +17005,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="103" spans="2:5">
+    <row r="103" spans="1:5">
+      <c r="A103">
+        <v>102</v>
+      </c>
       <c r="B103" t="s">
         <v>408</v>
       </c>
@@ -16860,7 +17022,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="104" spans="2:5">
+    <row r="104" spans="1:5">
+      <c r="A104">
+        <v>103</v>
+      </c>
       <c r="B104" t="s">
         <v>409</v>
       </c>
@@ -16874,7 +17039,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="105" spans="2:5">
+    <row r="105" spans="1:5">
+      <c r="A105">
+        <v>104</v>
+      </c>
       <c r="B105" t="s">
         <v>410</v>
       </c>
@@ -16888,7 +17056,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="106" spans="2:5">
+    <row r="106" spans="1:5">
+      <c r="A106">
+        <v>105</v>
+      </c>
       <c r="B106" t="s">
         <v>411</v>
       </c>
@@ -16902,7 +17073,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="107" spans="2:5">
+    <row r="107" spans="1:5">
+      <c r="A107">
+        <v>106</v>
+      </c>
       <c r="B107" t="s">
         <v>412</v>
       </c>
@@ -16916,7 +17090,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="108" spans="2:5">
+    <row r="108" spans="1:5">
+      <c r="A108">
+        <v>107</v>
+      </c>
       <c r="B108" t="s">
         <v>413</v>
       </c>
@@ -16930,7 +17107,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="109" spans="2:5">
+    <row r="109" spans="1:5">
+      <c r="A109">
+        <v>108</v>
+      </c>
       <c r="B109" t="s">
         <v>414</v>
       </c>
@@ -16944,7 +17124,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="110" spans="2:5">
+    <row r="110" spans="1:5">
+      <c r="A110">
+        <v>109</v>
+      </c>
       <c r="B110" t="s">
         <v>415</v>
       </c>
@@ -16958,7 +17141,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="111" spans="2:5">
+    <row r="111" spans="1:5">
+      <c r="A111">
+        <v>110</v>
+      </c>
       <c r="B111" t="s">
         <v>416</v>
       </c>
@@ -16972,7 +17158,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="112" spans="2:5">
+    <row r="112" spans="1:5">
+      <c r="A112">
+        <v>111</v>
+      </c>
       <c r="B112" t="s">
         <v>417</v>
       </c>
@@ -16986,7 +17175,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="113" spans="2:5">
+    <row r="113" spans="1:5">
+      <c r="A113">
+        <v>112</v>
+      </c>
       <c r="B113" t="s">
         <v>418</v>
       </c>
@@ -17000,7 +17192,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="114" spans="2:5">
+    <row r="114" spans="1:5">
+      <c r="A114">
+        <v>113</v>
+      </c>
       <c r="B114" t="s">
         <v>419</v>
       </c>
@@ -17014,7 +17209,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="115" spans="2:5">
+    <row r="115" spans="1:5">
+      <c r="A115">
+        <v>114</v>
+      </c>
       <c r="B115" t="s">
         <v>420</v>
       </c>
@@ -17028,7 +17226,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="116" spans="2:5">
+    <row r="116" spans="1:5">
+      <c r="A116">
+        <v>115</v>
+      </c>
       <c r="B116" t="s">
         <v>421</v>
       </c>
@@ -17042,7 +17243,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="117" spans="2:5">
+    <row r="117" spans="1:5">
+      <c r="A117">
+        <v>116</v>
+      </c>
       <c r="B117" t="s">
         <v>422</v>
       </c>
@@ -17056,7 +17260,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="118" spans="2:5">
+    <row r="118" spans="1:5">
+      <c r="A118">
+        <v>117</v>
+      </c>
       <c r="B118" t="s">
         <v>423</v>
       </c>
@@ -17070,7 +17277,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="119" spans="2:5">
+    <row r="119" spans="1:5">
+      <c r="A119">
+        <v>118</v>
+      </c>
       <c r="B119" t="s">
         <v>424</v>
       </c>
@@ -17084,7 +17294,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="120" spans="2:5">
+    <row r="120" spans="1:5">
+      <c r="A120">
+        <v>119</v>
+      </c>
       <c r="B120" t="s">
         <v>425</v>
       </c>
@@ -17098,7 +17311,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="121" spans="2:5">
+    <row r="121" spans="1:5">
+      <c r="A121">
+        <v>120</v>
+      </c>
       <c r="B121" t="s">
         <v>426</v>
       </c>
@@ -17112,7 +17328,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="122" spans="2:5">
+    <row r="122" spans="1:5">
+      <c r="A122">
+        <v>121</v>
+      </c>
       <c r="B122" t="s">
         <v>427</v>
       </c>
@@ -17126,7 +17345,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="123" spans="2:5">
+    <row r="123" spans="1:5">
+      <c r="A123">
+        <v>122</v>
+      </c>
       <c r="B123" t="s">
         <v>428</v>
       </c>
@@ -17140,7 +17362,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="124" spans="2:5">
+    <row r="124" spans="1:5">
+      <c r="A124">
+        <v>123</v>
+      </c>
       <c r="B124" t="s">
         <v>429</v>
       </c>
@@ -17154,7 +17379,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="125" spans="2:5">
+    <row r="125" spans="1:5">
+      <c r="A125">
+        <v>124</v>
+      </c>
       <c r="B125" t="s">
         <v>430</v>
       </c>
@@ -17168,7 +17396,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="126" spans="2:5">
+    <row r="126" spans="1:5">
+      <c r="A126">
+        <v>125</v>
+      </c>
       <c r="B126" t="s">
         <v>431</v>
       </c>
@@ -17182,7 +17413,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="127" spans="2:5">
+    <row r="127" spans="1:5">
+      <c r="A127">
+        <v>126</v>
+      </c>
       <c r="B127" t="s">
         <v>432</v>
       </c>
@@ -17196,7 +17430,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="128" spans="2:5">
+    <row r="128" spans="1:5">
+      <c r="A128">
+        <v>127</v>
+      </c>
       <c r="B128" t="s">
         <v>433</v>
       </c>
@@ -17210,7 +17447,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="129" spans="2:5">
+    <row r="129" spans="1:5">
+      <c r="A129">
+        <v>128</v>
+      </c>
       <c r="B129" t="s">
         <v>434</v>
       </c>
@@ -17224,7 +17464,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="130" spans="2:5">
+    <row r="130" spans="1:5">
+      <c r="A130">
+        <v>129</v>
+      </c>
       <c r="B130" t="s">
         <v>435</v>
       </c>
@@ -17238,7 +17481,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="131" spans="2:5">
+    <row r="131" spans="1:5">
+      <c r="A131">
+        <v>130</v>
+      </c>
       <c r="B131" t="s">
         <v>436</v>
       </c>
@@ -17252,7 +17498,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="132" spans="2:5">
+    <row r="132" spans="1:5">
+      <c r="A132">
+        <v>131</v>
+      </c>
       <c r="B132" t="s">
         <v>437</v>
       </c>
@@ -17266,7 +17515,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="133" spans="2:5">
+    <row r="133" spans="1:5">
+      <c r="A133">
+        <v>132</v>
+      </c>
       <c r="B133" t="s">
         <v>438</v>
       </c>
@@ -17280,7 +17532,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="134" spans="2:5">
+    <row r="134" spans="1:5">
+      <c r="A134">
+        <v>133</v>
+      </c>
       <c r="B134" t="s">
         <v>439</v>
       </c>
@@ -17294,7 +17549,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="135" spans="2:5">
+    <row r="135" spans="1:5">
+      <c r="A135">
+        <v>134</v>
+      </c>
       <c r="B135" t="s">
         <v>440</v>
       </c>
@@ -17308,7 +17566,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="136" spans="2:5">
+    <row r="136" spans="1:5">
+      <c r="A136">
+        <v>135</v>
+      </c>
       <c r="B136" t="s">
         <v>441</v>
       </c>
@@ -17322,7 +17583,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="137" spans="2:5">
+    <row r="137" spans="1:5">
+      <c r="A137">
+        <v>136</v>
+      </c>
       <c r="B137" t="s">
         <v>442</v>
       </c>
@@ -17336,7 +17600,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="138" spans="2:5">
+    <row r="138" spans="1:5">
+      <c r="A138">
+        <v>137</v>
+      </c>
       <c r="B138" t="s">
         <v>443</v>
       </c>
@@ -17350,7 +17617,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="139" spans="2:5">
+    <row r="139" spans="1:5">
+      <c r="A139">
+        <v>138</v>
+      </c>
       <c r="B139" t="s">
         <v>444</v>
       </c>
@@ -17364,7 +17634,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="140" spans="2:5">
+    <row r="140" spans="1:5">
+      <c r="A140">
+        <v>139</v>
+      </c>
       <c r="B140" t="s">
         <v>445</v>
       </c>
@@ -17378,7 +17651,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="141" spans="2:5">
+    <row r="141" spans="1:5">
+      <c r="A141">
+        <v>140</v>
+      </c>
       <c r="B141" t="s">
         <v>446</v>
       </c>
@@ -17392,7 +17668,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="142" spans="2:5">
+    <row r="142" spans="1:5">
+      <c r="A142">
+        <v>141</v>
+      </c>
       <c r="B142" t="s">
         <v>447</v>
       </c>
@@ -17406,7 +17685,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="143" spans="2:5">
+    <row r="143" spans="1:5">
+      <c r="A143">
+        <v>142</v>
+      </c>
       <c r="B143" t="s">
         <v>448</v>
       </c>
@@ -17420,7 +17702,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="144" spans="2:5">
+    <row r="144" spans="1:5">
+      <c r="A144">
+        <v>143</v>
+      </c>
       <c r="B144" t="s">
         <v>449</v>
       </c>
@@ -17434,7 +17719,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="145" spans="2:5">
+    <row r="145" spans="1:5">
+      <c r="A145">
+        <v>144</v>
+      </c>
       <c r="B145" t="s">
         <v>450</v>
       </c>
@@ -17448,7 +17736,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="146" spans="2:5">
+    <row r="146" spans="1:5">
+      <c r="A146">
+        <v>145</v>
+      </c>
       <c r="B146" t="s">
         <v>451</v>
       </c>
@@ -17462,7 +17753,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="147" spans="2:5">
+    <row r="147" spans="1:5">
+      <c r="A147">
+        <v>146</v>
+      </c>
       <c r="B147" t="s">
         <v>452</v>
       </c>
@@ -17476,7 +17770,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="148" spans="2:5">
+    <row r="148" spans="1:5">
+      <c r="A148">
+        <v>147</v>
+      </c>
       <c r="B148" t="s">
         <v>453</v>
       </c>
@@ -17490,7 +17787,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="149" spans="2:5">
+    <row r="149" spans="1:5">
+      <c r="A149">
+        <v>148</v>
+      </c>
       <c r="B149" t="s">
         <v>454</v>
       </c>
@@ -17504,7 +17804,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="150" spans="2:5">
+    <row r="150" spans="1:5">
+      <c r="A150">
+        <v>149</v>
+      </c>
       <c r="B150" t="s">
         <v>455</v>
       </c>
@@ -17518,7 +17821,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="151" spans="2:5">
+    <row r="151" spans="1:5">
+      <c r="A151">
+        <v>150</v>
+      </c>
       <c r="B151" t="s">
         <v>456</v>
       </c>
@@ -17532,7 +17838,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="152" spans="2:5">
+    <row r="152" spans="1:5">
+      <c r="A152">
+        <v>151</v>
+      </c>
       <c r="B152" t="s">
         <v>457</v>
       </c>
@@ -17546,7 +17855,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="153" spans="2:5">
+    <row r="153" spans="1:5">
+      <c r="A153">
+        <v>152</v>
+      </c>
       <c r="B153" t="s">
         <v>458</v>
       </c>
@@ -17560,7 +17872,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="154" spans="2:5">
+    <row r="154" spans="1:5">
+      <c r="A154">
+        <v>153</v>
+      </c>
       <c r="B154" t="s">
         <v>459</v>
       </c>
@@ -17574,7 +17889,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="155" spans="2:5">
+    <row r="155" spans="1:5">
+      <c r="A155">
+        <v>154</v>
+      </c>
       <c r="B155" t="s">
         <v>460</v>
       </c>
@@ -17588,7 +17906,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="156" spans="2:5">
+    <row r="156" spans="1:5">
+      <c r="A156">
+        <v>155</v>
+      </c>
       <c r="B156" t="s">
         <v>461</v>
       </c>
@@ -17602,7 +17923,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="157" spans="2:5">
+    <row r="157" spans="1:5">
+      <c r="A157">
+        <v>156</v>
+      </c>
       <c r="B157" t="s">
         <v>462</v>
       </c>
@@ -17616,7 +17940,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="158" spans="2:5">
+    <row r="158" spans="1:5">
+      <c r="A158">
+        <v>157</v>
+      </c>
       <c r="B158" t="s">
         <v>463</v>
       </c>
@@ -17630,7 +17957,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="159" spans="2:5">
+    <row r="159" spans="1:5">
+      <c r="A159">
+        <v>158</v>
+      </c>
       <c r="B159" t="s">
         <v>464</v>
       </c>
@@ -17644,7 +17974,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="160" spans="2:5">
+    <row r="160" spans="1:5">
+      <c r="A160">
+        <v>159</v>
+      </c>
       <c r="B160" t="s">
         <v>465</v>
       </c>
@@ -17658,7 +17991,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="161" spans="2:5">
+    <row r="161" spans="1:5">
+      <c r="A161">
+        <v>160</v>
+      </c>
       <c r="B161" t="s">
         <v>466</v>
       </c>
@@ -17672,7 +18008,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="162" spans="2:5">
+    <row r="162" spans="1:5">
+      <c r="A162">
+        <v>161</v>
+      </c>
       <c r="B162" t="s">
         <v>467</v>
       </c>
@@ -17686,7 +18025,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="163" spans="2:5">
+    <row r="163" spans="1:5">
+      <c r="A163">
+        <v>162</v>
+      </c>
       <c r="B163" t="s">
         <v>468</v>
       </c>
@@ -17700,7 +18042,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="164" spans="2:5">
+    <row r="164" spans="1:5">
+      <c r="A164">
+        <v>163</v>
+      </c>
       <c r="B164" t="s">
         <v>469</v>
       </c>
@@ -17714,7 +18059,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="165" spans="2:5">
+    <row r="165" spans="1:5">
+      <c r="A165">
+        <v>164</v>
+      </c>
       <c r="B165" t="s">
         <v>470</v>
       </c>
@@ -17728,7 +18076,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="166" spans="2:5">
+    <row r="166" spans="1:5">
+      <c r="A166">
+        <v>165</v>
+      </c>
       <c r="B166" t="s">
         <v>471</v>
       </c>
@@ -17742,7 +18093,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="167" spans="2:5">
+    <row r="167" spans="1:5">
+      <c r="A167">
+        <v>166</v>
+      </c>
       <c r="B167" t="s">
         <v>472</v>
       </c>
@@ -17756,7 +18110,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="168" spans="2:5">
+    <row r="168" spans="1:5">
+      <c r="A168">
+        <v>167</v>
+      </c>
       <c r="B168" t="s">
         <v>473</v>
       </c>
@@ -17770,7 +18127,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="169" spans="2:5">
+    <row r="169" spans="1:5">
+      <c r="A169">
+        <v>168</v>
+      </c>
       <c r="B169" t="s">
         <v>474</v>
       </c>
@@ -17784,7 +18144,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="170" spans="2:5">
+    <row r="170" spans="1:5">
+      <c r="A170">
+        <v>169</v>
+      </c>
       <c r="B170" t="s">
         <v>475</v>
       </c>
@@ -17798,7 +18161,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="171" spans="2:5">
+    <row r="171" spans="1:5">
+      <c r="A171">
+        <v>170</v>
+      </c>
       <c r="B171" t="s">
         <v>476</v>
       </c>
@@ -17812,7 +18178,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="172" spans="2:5">
+    <row r="172" spans="1:5">
+      <c r="A172">
+        <v>171</v>
+      </c>
       <c r="B172" t="s">
         <v>477</v>
       </c>
@@ -17826,7 +18195,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="173" spans="2:5">
+    <row r="173" spans="1:5">
+      <c r="A173">
+        <v>172</v>
+      </c>
       <c r="B173" t="s">
         <v>478</v>
       </c>
@@ -17840,7 +18212,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="174" spans="2:5">
+    <row r="174" spans="1:5">
+      <c r="A174">
+        <v>173</v>
+      </c>
       <c r="B174" t="s">
         <v>479</v>
       </c>
@@ -17854,7 +18229,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="175" spans="2:5">
+    <row r="175" spans="1:5">
+      <c r="A175">
+        <v>174</v>
+      </c>
       <c r="B175" t="s">
         <v>480</v>
       </c>
@@ -17868,7 +18246,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="176" spans="2:5">
+    <row r="176" spans="1:5">
+      <c r="A176">
+        <v>175</v>
+      </c>
       <c r="B176" t="s">
         <v>481</v>
       </c>
@@ -17882,7 +18263,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="177" spans="2:5">
+    <row r="177" spans="1:5">
+      <c r="A177">
+        <v>176</v>
+      </c>
       <c r="B177" t="s">
         <v>482</v>
       </c>
@@ -17896,7 +18280,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="178" spans="2:5">
+    <row r="178" spans="1:5">
+      <c r="A178">
+        <v>177</v>
+      </c>
       <c r="B178" t="s">
         <v>483</v>
       </c>
@@ -17910,7 +18297,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="179" spans="2:5">
+    <row r="179" spans="1:5">
+      <c r="A179">
+        <v>178</v>
+      </c>
       <c r="B179" t="s">
         <v>484</v>
       </c>
@@ -17924,7 +18314,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="180" spans="2:5">
+    <row r="180" spans="1:5">
+      <c r="A180">
+        <v>179</v>
+      </c>
       <c r="B180" t="s">
         <v>485</v>
       </c>
@@ -17938,7 +18331,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="181" spans="2:5">
+    <row r="181" spans="1:5">
+      <c r="A181">
+        <v>180</v>
+      </c>
       <c r="B181" t="s">
         <v>486</v>
       </c>
@@ -17952,7 +18348,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="182" spans="2:5">
+    <row r="182" spans="1:5">
+      <c r="A182">
+        <v>181</v>
+      </c>
       <c r="B182" t="s">
         <v>487</v>
       </c>
@@ -17966,7 +18365,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="183" spans="2:5">
+    <row r="183" spans="1:5">
+      <c r="A183">
+        <v>182</v>
+      </c>
       <c r="B183" t="s">
         <v>488</v>
       </c>
@@ -17980,7 +18382,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="184" spans="2:5">
+    <row r="184" spans="1:5">
+      <c r="A184">
+        <v>183</v>
+      </c>
       <c r="B184" t="s">
         <v>489</v>
       </c>
@@ -17994,7 +18399,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="185" spans="2:5">
+    <row r="185" spans="1:5">
+      <c r="A185">
+        <v>184</v>
+      </c>
       <c r="B185" t="s">
         <v>490</v>
       </c>
@@ -18008,7 +18416,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="186" spans="2:5">
+    <row r="186" spans="1:5">
+      <c r="A186">
+        <v>185</v>
+      </c>
       <c r="B186" t="s">
         <v>491</v>
       </c>
@@ -18022,7 +18433,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="187" spans="2:5">
+    <row r="187" spans="1:5">
+      <c r="A187">
+        <v>186</v>
+      </c>
       <c r="B187" t="s">
         <v>492</v>
       </c>
@@ -18036,7 +18450,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="188" spans="2:5">
+    <row r="188" spans="1:5">
+      <c r="A188">
+        <v>187</v>
+      </c>
       <c r="B188" t="s">
         <v>493</v>
       </c>
@@ -18050,7 +18467,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="189" spans="2:5">
+    <row r="189" spans="1:5">
+      <c r="A189">
+        <v>188</v>
+      </c>
       <c r="B189" t="s">
         <v>494</v>
       </c>
@@ -18064,7 +18484,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="190" spans="2:5">
+    <row r="190" spans="1:5">
+      <c r="A190">
+        <v>189</v>
+      </c>
       <c r="B190" t="s">
         <v>495</v>
       </c>
@@ -18078,7 +18501,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="191" spans="2:5">
+    <row r="191" spans="1:5">
+      <c r="A191">
+        <v>190</v>
+      </c>
       <c r="B191" t="s">
         <v>496</v>
       </c>
@@ -18092,7 +18518,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="192" spans="2:5">
+    <row r="192" spans="1:5">
+      <c r="A192">
+        <v>191</v>
+      </c>
       <c r="B192" t="s">
         <v>497</v>
       </c>
@@ -18106,7 +18535,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="193" spans="2:5">
+    <row r="193" spans="1:5">
+      <c r="A193">
+        <v>192</v>
+      </c>
       <c r="B193" t="s">
         <v>498</v>
       </c>
@@ -18120,7 +18552,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="194" spans="2:5">
+    <row r="194" spans="1:5">
+      <c r="A194">
+        <v>193</v>
+      </c>
       <c r="B194" t="s">
         <v>499</v>
       </c>
@@ -18134,7 +18569,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="195" spans="2:5">
+    <row r="195" spans="1:5">
+      <c r="A195">
+        <v>194</v>
+      </c>
       <c r="B195" t="s">
         <v>500</v>
       </c>
@@ -18148,7 +18586,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="196" spans="2:5">
+    <row r="196" spans="1:5">
+      <c r="A196">
+        <v>195</v>
+      </c>
       <c r="B196" t="s">
         <v>501</v>
       </c>
@@ -18162,7 +18603,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="197" spans="2:5">
+    <row r="197" spans="1:5">
+      <c r="A197">
+        <v>196</v>
+      </c>
       <c r="B197" t="s">
         <v>502</v>
       </c>
@@ -18176,7 +18620,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="198" spans="2:5">
+    <row r="198" spans="1:5">
+      <c r="A198">
+        <v>197</v>
+      </c>
       <c r="B198" t="s">
         <v>503</v>
       </c>
@@ -18190,7 +18637,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="199" spans="2:5">
+    <row r="199" spans="1:5">
+      <c r="A199">
+        <v>198</v>
+      </c>
       <c r="B199" t="s">
         <v>504</v>
       </c>
@@ -18204,7 +18654,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="200" spans="2:5">
+    <row r="200" spans="1:5">
+      <c r="A200">
+        <v>199</v>
+      </c>
       <c r="B200" t="s">
         <v>505</v>
       </c>
@@ -18218,7 +18671,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="201" spans="2:5">
+    <row r="201" spans="1:5">
+      <c r="A201">
+        <v>200</v>
+      </c>
       <c r="B201" t="s">
         <v>506</v>
       </c>
@@ -18232,7 +18688,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="202" spans="2:5">
+    <row r="202" spans="1:5">
+      <c r="A202">
+        <v>201</v>
+      </c>
       <c r="B202" t="s">
         <v>507</v>
       </c>
@@ -18246,7 +18705,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="203" spans="2:5">
+    <row r="203" spans="1:5">
+      <c r="A203">
+        <v>202</v>
+      </c>
       <c r="B203" t="s">
         <v>508</v>
       </c>
@@ -18260,7 +18722,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="204" spans="2:5">
+    <row r="204" spans="1:5">
+      <c r="A204">
+        <v>203</v>
+      </c>
       <c r="B204" t="s">
         <v>509</v>
       </c>
@@ -18274,7 +18739,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="205" spans="2:5">
+    <row r="205" spans="1:5">
+      <c r="A205">
+        <v>204</v>
+      </c>
       <c r="B205" t="s">
         <v>510</v>
       </c>
@@ -18288,7 +18756,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="206" spans="2:5">
+    <row r="206" spans="1:5">
+      <c r="A206">
+        <v>205</v>
+      </c>
       <c r="B206" t="s">
         <v>511</v>
       </c>
@@ -18302,7 +18773,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="207" spans="2:5">
+    <row r="207" spans="1:5">
+      <c r="A207">
+        <v>206</v>
+      </c>
       <c r="B207" t="s">
         <v>512</v>
       </c>
@@ -18316,7 +18790,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="208" spans="2:5">
+    <row r="208" spans="1:5">
+      <c r="A208">
+        <v>207</v>
+      </c>
       <c r="B208" t="s">
         <v>513</v>
       </c>
@@ -18330,7 +18807,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="209" spans="2:5">
+    <row r="209" spans="1:5">
+      <c r="A209">
+        <v>208</v>
+      </c>
       <c r="B209" t="s">
         <v>514</v>
       </c>
@@ -18344,7 +18824,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="210" spans="2:5">
+    <row r="210" spans="1:5">
+      <c r="A210">
+        <v>209</v>
+      </c>
       <c r="B210" t="s">
         <v>515</v>
       </c>
@@ -18358,7 +18841,10 @@
         <v>46013</v>
       </c>
     </row>
-    <row r="211" spans="2:5">
+    <row r="211" spans="1:5">
+      <c r="A211">
+        <v>210</v>
+      </c>
       <c r="B211" t="s">
         <v>516</v>
       </c>

</xml_diff>